<commit_message>
Add full formatting support: font, alignment, fill, border, number format, merged cells
- Font: name, color, underline, strikethrough (added to size/bold/italic)
- Alignment: horizontal, vertical, wrap_text
- Fill: solid background color
- Border: line style and color for all 4 sides
- Number format: preserve Excel format strings
- Merged cells: copy merge ranges and skip non-topleft cells on write/verify

https://claude.ai/code/session_0179fduQDX21vgHwbjCgDbza
</commit_message>
<xml_diff>
--- a/font_test.xlsx
+++ b/font_test.xlsx
@@ -26,15 +26,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <strike val="0"/>
       <sz val="18"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <strike val="0"/>
       <sz val="12"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <strike val="0"/>
       <sz val="10"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <strike val="0"/>
       <sz val="8"/>
     </font>
   </fonts>
@@ -46,7 +54,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -54,16 +62,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>

</xml_diff>